<commit_message>
Fix the original PSMBench project and update evaluation results
1.The original PSMBench project loss some fsm files (the fsm files related "qwen3:32b" and "gemma3:27b" is missing.). The reason is that Windows system do not use ":" in the file name. So I download again and change the file name which have ":" to "_".
2. Add the run_original_psmbench_evaluation.py to run the original PSMBench evaluation modules.
3. Update the PSMBench evaluation results.
4. Add the related dir path in the path.py
5.Change  the original PSMBench name: "PSMBench"-> "RFC_PSM_Benchmark-main"
</commit_message>
<xml_diff>
--- a/PSMBench_evaluation_results/states_match_results.xlsx
+++ b/PSMBench_evaluation_results/states_match_results.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21555" windowHeight="10365"/>
+    <workbookView windowHeight="17655"/>
   </bookViews>
   <sheets>
     <sheet name="states_match_results" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="31">
   <si>
     <t>Protocol</t>
   </si>
@@ -72,6 +72,12 @@
   </si>
   <si>
     <t>QWQ</t>
+  </si>
+  <si>
+    <t>QWen3</t>
+  </si>
+  <si>
+    <t>Gemma3</t>
   </si>
   <si>
     <t>Mistral</t>
@@ -1266,7 +1272,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H99"/>
+  <dimension ref="A1:H127"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="9.375" customWidth="1"/>
@@ -1469,85 +1475,85 @@
         <v>15</v>
       </c>
       <c r="C8">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D8">
         <v>5</v>
       </c>
       <c r="E8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8">
-        <v>0.4</v>
+        <v>0.75</v>
       </c>
       <c r="G8">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="H8">
-        <v>0.533</v>
+        <v>0.667</v>
       </c>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
       <c r="C9">
+        <v>10</v>
+      </c>
+      <c r="D9">
+        <v>5</v>
+      </c>
+      <c r="E9">
         <v>4</v>
       </c>
-      <c r="D9">
-        <v>3</v>
-      </c>
-      <c r="E9">
-        <v>3</v>
-      </c>
       <c r="F9">
-        <v>0.75</v>
+        <v>0.4</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H9">
-        <v>0.857</v>
+        <v>0.533</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C10">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F10">
-        <v>0.214</v>
+        <v>0.4</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H10">
-        <v>0.353</v>
+        <v>0.533</v>
       </c>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D11">
         <v>3</v>
@@ -1556,24 +1562,24 @@
         <v>3</v>
       </c>
       <c r="F11">
-        <v>0.6</v>
+        <v>0.75</v>
       </c>
       <c r="G11">
         <v>1</v>
       </c>
       <c r="H11">
-        <v>0.75</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C12">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="D12">
         <v>3</v>
@@ -1582,21 +1588,21 @@
         <v>3</v>
       </c>
       <c r="F12">
-        <v>0.75</v>
+        <v>0.214</v>
       </c>
       <c r="G12">
         <v>1</v>
       </c>
       <c r="H12">
-        <v>0.857</v>
+        <v>0.353</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C13">
         <v>5</v>
@@ -1619,10 +1625,10 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C14">
         <v>4</v>
@@ -1631,27 +1637,27 @@
         <v>3</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F14">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="G14">
-        <v>0.333</v>
+        <v>1</v>
       </c>
       <c r="H14">
-        <v>0.286</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C15">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="D15">
         <v>3</v>
@@ -1660,559 +1666,559 @@
         <v>3</v>
       </c>
       <c r="F15">
-        <v>0.25</v>
+        <v>0.6</v>
       </c>
       <c r="G15">
         <v>1</v>
       </c>
       <c r="H15">
-        <v>0.4</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C16">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D16">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E16">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F16">
-        <v>1.143</v>
+        <v>0.25</v>
       </c>
       <c r="G16">
-        <v>0.667</v>
+        <v>0.333</v>
       </c>
       <c r="H16">
-        <v>0.842</v>
+        <v>0.286</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C17">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="D17">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E17">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="F17">
-        <v>0.458</v>
+        <v>0.75</v>
       </c>
       <c r="G17">
-        <v>0.917</v>
+        <v>1</v>
       </c>
       <c r="H17">
-        <v>0.611</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18">
         <v>17</v>
       </c>
-      <c r="B18" t="s">
-        <v>11</v>
-      </c>
-      <c r="C18">
-        <v>11</v>
-      </c>
       <c r="D18">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E18">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F18">
-        <v>0.455</v>
+        <v>0.176</v>
       </c>
       <c r="G18">
-        <v>0.417</v>
+        <v>1</v>
       </c>
       <c r="H18">
-        <v>0.435</v>
+        <v>0.299</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
         <v>17</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19">
         <v>12</v>
       </c>
-      <c r="C19">
-        <v>26</v>
-      </c>
       <c r="D19">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E19">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F19">
-        <v>0.385</v>
+        <v>0.25</v>
       </c>
       <c r="G19">
-        <v>0.833</v>
+        <v>1</v>
       </c>
       <c r="H19">
-        <v>0.527</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C20">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D20">
         <v>12</v>
       </c>
       <c r="E20">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F20">
-        <v>1.25</v>
+        <v>1.143</v>
       </c>
       <c r="G20">
-        <v>0.417</v>
+        <v>0.667</v>
       </c>
       <c r="H20">
-        <v>0.625</v>
+        <v>0.842</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C21">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="D21">
         <v>12</v>
       </c>
       <c r="E21">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F21">
-        <v>0.571</v>
+        <v>0.458</v>
       </c>
       <c r="G21">
-        <v>0.667</v>
+        <v>0.917</v>
       </c>
       <c r="H21">
-        <v>0.615</v>
+        <v>0.611</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B22" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C22">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D22">
         <v>12</v>
       </c>
       <c r="E22">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F22">
-        <v>0.55</v>
+        <v>0.455</v>
       </c>
       <c r="G22">
-        <v>0.917</v>
+        <v>0.417</v>
       </c>
       <c r="H22">
-        <v>0.688</v>
+        <v>0.435</v>
       </c>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B23" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C23">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D23">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E23">
         <v>10</v>
       </c>
       <c r="F23">
-        <v>0.667</v>
+        <v>0.385</v>
       </c>
       <c r="G23">
-        <v>1</v>
+        <v>0.833</v>
       </c>
       <c r="H23">
-        <v>0.8</v>
+        <v>0.527</v>
       </c>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B24" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C24">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D24">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E24">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F24">
-        <v>0.526</v>
+        <v>1.25</v>
       </c>
       <c r="G24">
-        <v>1</v>
+        <v>0.417</v>
       </c>
       <c r="H24">
-        <v>0.689</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="25" spans="1:8">
       <c r="A25" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B25" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C25">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D25">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E25">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F25">
+        <v>0.571</v>
+      </c>
+      <c r="G25">
         <v>0.667</v>
       </c>
-      <c r="G25">
-        <v>1</v>
-      </c>
       <c r="H25">
-        <v>0.8</v>
+        <v>0.615</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B26" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26">
+        <v>7</v>
+      </c>
+      <c r="D26">
         <v>12</v>
       </c>
-      <c r="C26">
-        <v>13</v>
-      </c>
-      <c r="D26">
-        <v>10</v>
-      </c>
       <c r="E26">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F26">
-        <v>0.769</v>
+        <v>0.714</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>0.417</v>
       </c>
       <c r="H26">
-        <v>0.869</v>
+        <v>0.527</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C27">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D27">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E27">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F27">
-        <v>0.667</v>
+        <v>0.455</v>
       </c>
       <c r="G27">
-        <v>1</v>
+        <v>0.417</v>
       </c>
       <c r="H27">
-        <v>0.8</v>
+        <v>0.435</v>
       </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B28" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C28">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="D28">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E28">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="F28">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
       <c r="G28">
-        <v>0.3</v>
+        <v>0.917</v>
       </c>
       <c r="H28">
-        <v>0.4</v>
+        <v>0.688</v>
       </c>
     </row>
     <row r="29" spans="1:8">
       <c r="A29" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29">
         <v>15</v>
       </c>
-      <c r="C29">
-        <v>9</v>
-      </c>
       <c r="D29">
         <v>10</v>
       </c>
       <c r="E29">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F29">
-        <v>0.222</v>
+        <v>0.667</v>
       </c>
       <c r="G29">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="H29">
-        <v>0.21</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="30" spans="1:8">
       <c r="A30" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" t="s">
+        <v>10</v>
+      </c>
+      <c r="C30">
         <v>19</v>
       </c>
-      <c r="B30" t="s">
-        <v>9</v>
-      </c>
-      <c r="C30">
-        <v>8</v>
-      </c>
       <c r="D30">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E30">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>0.526</v>
       </c>
       <c r="G30">
-        <v>0.889</v>
+        <v>1</v>
       </c>
       <c r="H30">
-        <v>0.941</v>
+        <v>0.689</v>
       </c>
     </row>
     <row r="31" spans="1:8">
       <c r="A31" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B31" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C31">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D31">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E31">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F31">
-        <v>0.3</v>
+        <v>0.667</v>
       </c>
       <c r="G31">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="H31">
-        <v>0.414</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B32" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C32">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D32">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E32">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F32">
-        <v>0.333</v>
+        <v>0.769</v>
       </c>
       <c r="G32">
-        <v>0.556</v>
+        <v>1</v>
       </c>
       <c r="H32">
-        <v>0.417</v>
+        <v>0.869</v>
       </c>
     </row>
     <row r="33" spans="1:8">
       <c r="A33" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B33" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C33">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D33">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>0.667</v>
       </c>
       <c r="G33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B34" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C34">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="D34">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E34">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F34">
-        <v>0.667</v>
+        <v>0.6</v>
       </c>
       <c r="G34">
-        <v>0.889</v>
+        <v>0.3</v>
       </c>
       <c r="H34">
-        <v>0.762</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B35" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C35">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="D35">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E35">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F35">
-        <v>1.667</v>
+        <v>0.545</v>
       </c>
       <c r="G35">
-        <v>0.556</v>
+        <v>0.6</v>
       </c>
       <c r="H35">
-        <v>0.834</v>
+        <v>0.571</v>
       </c>
     </row>
     <row r="36" spans="1:8">
       <c r="A36" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B36" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C36">
         <v>6</v>
       </c>
       <c r="D36">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E36">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F36">
-        <v>1</v>
+        <v>0.333</v>
       </c>
       <c r="G36">
-        <v>0.667</v>
+        <v>0.2</v>
       </c>
       <c r="H36">
-        <v>0.8</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -2220,181 +2226,181 @@
         <v>20</v>
       </c>
       <c r="B37" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C37">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D37">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E37">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F37">
-        <v>1</v>
+        <v>0.222</v>
       </c>
       <c r="G37">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="H37">
-        <v>1</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="38" spans="1:8">
       <c r="A38" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B38" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C38">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D38">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E38">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F38">
-        <v>0.462</v>
+        <v>1</v>
       </c>
       <c r="G38">
-        <v>1</v>
+        <v>0.889</v>
       </c>
       <c r="H38">
-        <v>0.632</v>
+        <v>0.941</v>
       </c>
     </row>
     <row r="39" spans="1:8">
       <c r="A39" t="s">
+        <v>21</v>
+      </c>
+      <c r="B39" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39">
         <v>20</v>
       </c>
-      <c r="B39" t="s">
-        <v>11</v>
-      </c>
-      <c r="C39">
-        <v>8</v>
-      </c>
       <c r="D39">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E39">
         <v>6</v>
       </c>
       <c r="F39">
-        <v>0.75</v>
+        <v>0.3</v>
       </c>
       <c r="G39">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="H39">
-        <v>0.857</v>
+        <v>0.414</v>
       </c>
     </row>
     <row r="40" spans="1:8">
       <c r="A40" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B40" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C40">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D40">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E40">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F40">
-        <v>0.667</v>
+        <v>0.333</v>
       </c>
       <c r="G40">
-        <v>1</v>
+        <v>0.556</v>
       </c>
       <c r="H40">
-        <v>0.8</v>
+        <v>0.417</v>
       </c>
     </row>
     <row r="41" spans="1:8">
       <c r="A41" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C41">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D41">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E41">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H41">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:8">
       <c r="A42" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B42" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C42">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D42">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E42">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F42">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>0.889</v>
       </c>
       <c r="H42">
-        <v>1</v>
+        <v>0.762</v>
       </c>
     </row>
     <row r="43" spans="1:8">
       <c r="A43" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B43" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C43">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D43">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E43">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F43">
-        <v>0.3</v>
+        <v>1.667</v>
       </c>
       <c r="G43">
-        <v>0.5</v>
+        <v>0.556</v>
       </c>
       <c r="H43">
-        <v>0.375</v>
+        <v>0.834</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -2402,25 +2408,25 @@
         <v>21</v>
       </c>
       <c r="B44" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="C44">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="D44">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E44">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F44">
-        <v>0.2</v>
+        <v>2</v>
       </c>
       <c r="G44">
-        <v>1</v>
+        <v>0.889</v>
       </c>
       <c r="H44">
-        <v>0.333</v>
+        <v>1.231</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -2428,25 +2434,25 @@
         <v>21</v>
       </c>
       <c r="B45" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C45">
-        <v>88</v>
+        <v>4</v>
       </c>
       <c r="D45">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E45">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F45">
-        <v>0.034</v>
+        <v>1.5</v>
       </c>
       <c r="G45">
-        <v>0.6</v>
+        <v>0.667</v>
       </c>
       <c r="H45">
-        <v>0.064</v>
+        <v>0.923</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -2454,129 +2460,129 @@
         <v>21</v>
       </c>
       <c r="B46" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C46">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="D46">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E46">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F46">
-        <v>0.116</v>
+        <v>1</v>
       </c>
       <c r="G46">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="H46">
-        <v>0.208</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="47" spans="1:8">
       <c r="A47" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B47" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C47">
-        <v>65</v>
+        <v>6</v>
       </c>
       <c r="D47">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E47">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F47">
-        <v>0.077</v>
+        <v>1</v>
       </c>
       <c r="G47">
         <v>1</v>
       </c>
       <c r="H47">
-        <v>0.143</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:8">
       <c r="A48" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B48" t="s">
+        <v>10</v>
+      </c>
+      <c r="C48">
         <v>13</v>
       </c>
-      <c r="C48">
-        <v>12</v>
-      </c>
       <c r="D48">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E48">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F48">
-        <v>0.417</v>
+        <v>0.462</v>
       </c>
       <c r="G48">
         <v>1</v>
       </c>
       <c r="H48">
-        <v>0.589</v>
+        <v>0.632</v>
       </c>
     </row>
     <row r="49" spans="1:8">
       <c r="A49" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B49" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C49">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D49">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E49">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F49">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="G49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H49">
-        <v>0</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="50" spans="1:8">
       <c r="A50" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B50" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C50">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D50">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E50">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F50">
-        <v>0.031</v>
+        <v>0.667</v>
       </c>
       <c r="G50">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="H50">
-        <v>0.054</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -2584,25 +2590,25 @@
         <v>22</v>
       </c>
       <c r="B51" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C51">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D51">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E51">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F51">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="G51">
         <v>1</v>
       </c>
       <c r="H51">
-        <v>0.75</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -2610,25 +2616,25 @@
         <v>22</v>
       </c>
       <c r="B52" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C52">
-        <v>47</v>
+        <v>6</v>
       </c>
       <c r="D52">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E52">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F52">
-        <v>0.064</v>
+        <v>1</v>
       </c>
       <c r="G52">
         <v>1</v>
       </c>
       <c r="H52">
-        <v>0.12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -2636,25 +2642,25 @@
         <v>22</v>
       </c>
       <c r="B53" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C53">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="D53">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E53">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F53">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="G53">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="H53">
-        <v>0.174</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -2662,25 +2668,25 @@
         <v>22</v>
       </c>
       <c r="B54" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C54">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="D54">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F54">
-        <v>0.118</v>
+        <v>0.857</v>
       </c>
       <c r="G54">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="H54">
-        <v>0.201</v>
+        <v>0.923</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -2688,77 +2694,77 @@
         <v>22</v>
       </c>
       <c r="B55" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C55">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D55">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E55">
         <v>3</v>
       </c>
       <c r="F55">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="G55">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H55">
-        <v>1</v>
+        <v>0.375</v>
       </c>
     </row>
     <row r="56" spans="1:8">
       <c r="A56" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B56" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C56">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="D56">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E56">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F56">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="G56">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H56">
-        <v>0</v>
+        <v>0.333</v>
       </c>
     </row>
     <row r="57" spans="1:8">
       <c r="A57" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B57" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C57">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="D57">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E57">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F57">
-        <v>0.045</v>
+        <v>0.034</v>
       </c>
       <c r="G57">
-        <v>0.333</v>
+        <v>0.6</v>
       </c>
       <c r="H57">
-        <v>0.079</v>
+        <v>0.064</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -2766,25 +2772,25 @@
         <v>23</v>
       </c>
       <c r="B58" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C58">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="D58">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E58">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F58">
-        <v>0.75</v>
+        <v>0.116</v>
       </c>
       <c r="G58">
         <v>1</v>
       </c>
       <c r="H58">
-        <v>0.857</v>
+        <v>0.208</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -2792,25 +2798,25 @@
         <v>23</v>
       </c>
       <c r="B59" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C59">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="D59">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E59">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F59">
-        <v>0.22</v>
+        <v>0.077</v>
       </c>
       <c r="G59">
         <v>1</v>
       </c>
       <c r="H59">
-        <v>0.361</v>
+        <v>0.143</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -2818,25 +2824,25 @@
         <v>23</v>
       </c>
       <c r="B60" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C60">
         <v>12</v>
       </c>
       <c r="D60">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E60">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F60">
-        <v>0.75</v>
+        <v>0.417</v>
       </c>
       <c r="G60">
         <v>1</v>
       </c>
       <c r="H60">
-        <v>0.857</v>
+        <v>0.589</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -2844,25 +2850,25 @@
         <v>23</v>
       </c>
       <c r="B61" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C61">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="D61">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E61">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F61">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="G61">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H61">
-        <v>0.621</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -2870,25 +2876,25 @@
         <v>23</v>
       </c>
       <c r="B62" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C62">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D62">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E62">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F62">
-        <v>0.75</v>
+        <v>0.182</v>
       </c>
       <c r="G62">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="H62">
-        <v>0.857</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -2896,25 +2902,25 @@
         <v>23</v>
       </c>
       <c r="B63" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C63">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="D63">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E63">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F63">
-        <v>1.5</v>
+        <v>0.074</v>
       </c>
       <c r="G63">
-        <v>0.667</v>
+        <v>0.4</v>
       </c>
       <c r="H63">
-        <v>0.923</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -2922,25 +2928,25 @@
         <v>23</v>
       </c>
       <c r="B64" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C64">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="D64">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E64">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F64">
+        <v>0.031</v>
+      </c>
+      <c r="G64">
         <v>0.2</v>
       </c>
-      <c r="G64">
-        <v>0.222</v>
-      </c>
       <c r="H64">
-        <v>0.21</v>
+        <v>0.054</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -2951,22 +2957,22 @@
         <v>9</v>
       </c>
       <c r="C65">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D65">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E65">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F65">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="G65">
         <v>1</v>
       </c>
       <c r="H65">
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -2977,22 +2983,22 @@
         <v>10</v>
       </c>
       <c r="C66">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="D66">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E66">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F66">
-        <v>0.727</v>
+        <v>0.064</v>
       </c>
       <c r="G66">
         <v>1</v>
       </c>
       <c r="H66">
-        <v>0.842</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -3003,22 +3009,22 @@
         <v>11</v>
       </c>
       <c r="C67">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="D67">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E67">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F67">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="G67">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="H67">
-        <v>1</v>
+        <v>0.174</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -3029,22 +3035,22 @@
         <v>12</v>
       </c>
       <c r="C68">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D68">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E68">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F68">
+        <v>0.118</v>
+      </c>
+      <c r="G68">
         <v>0.667</v>
       </c>
-      <c r="G68">
-        <v>0.5</v>
-      </c>
       <c r="H68">
-        <v>0.572</v>
+        <v>0.201</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -3055,22 +3061,22 @@
         <v>13</v>
       </c>
       <c r="C69">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D69">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E69">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F69">
-        <v>1.143</v>
+        <v>1</v>
       </c>
       <c r="G69">
         <v>1</v>
       </c>
       <c r="H69">
-        <v>1.067</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -3081,22 +3087,22 @@
         <v>14</v>
       </c>
       <c r="C70">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D70">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E70">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F70">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="G70">
-        <v>0.625</v>
+        <v>0</v>
       </c>
       <c r="H70">
-        <v>0.833</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -3110,71 +3116,71 @@
         <v>3</v>
       </c>
       <c r="D71">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E71">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F71">
-        <v>1.333</v>
+        <v>1</v>
       </c>
       <c r="G71">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H71">
-        <v>0.727</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72" spans="1:8">
       <c r="A72" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B72" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C72">
         <v>14</v>
       </c>
       <c r="D72">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E72">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F72">
-        <v>0.357</v>
+        <v>0.214</v>
       </c>
       <c r="G72">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H72">
-        <v>0.417</v>
+        <v>0.353</v>
       </c>
     </row>
     <row r="73" spans="1:8">
       <c r="A73" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B73" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C73">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="D73">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E73">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F73">
-        <v>0.146</v>
+        <v>0.045</v>
       </c>
       <c r="G73">
-        <v>0.6</v>
+        <v>0.333</v>
       </c>
       <c r="H73">
-        <v>0.235</v>
+        <v>0.079</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -3182,25 +3188,25 @@
         <v>25</v>
       </c>
       <c r="B74" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C74">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D74">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E74">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F74">
-        <v>0.143</v>
+        <v>0.75</v>
       </c>
       <c r="G74">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="H74">
-        <v>0.167</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="75" spans="1:8">
@@ -3208,25 +3214,25 @@
         <v>25</v>
       </c>
       <c r="B75" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C75">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="D75">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E75">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="F75">
-        <v>0.4</v>
+        <v>0.22</v>
       </c>
       <c r="G75">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H75">
-        <v>0.48</v>
+        <v>0.361</v>
       </c>
     </row>
     <row r="76" spans="1:8">
@@ -3234,25 +3240,25 @@
         <v>25</v>
       </c>
       <c r="B76" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C76">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="D76">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E76">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F76">
-        <v>0.348</v>
+        <v>0.75</v>
       </c>
       <c r="G76">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="H76">
-        <v>0.485</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="77" spans="1:8">
@@ -3260,25 +3266,25 @@
         <v>25</v>
       </c>
       <c r="B77" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C77">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="D77">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E77">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F77">
-        <v>0.833</v>
+        <v>0.45</v>
       </c>
       <c r="G77">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H77">
-        <v>0.625</v>
+        <v>0.621</v>
       </c>
     </row>
     <row r="78" spans="1:8">
@@ -3286,129 +3292,129 @@
         <v>25</v>
       </c>
       <c r="B78" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C78">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D78">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E78">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F78">
-        <v>0.2</v>
+        <v>0.75</v>
       </c>
       <c r="G78">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="H78">
-        <v>0.267</v>
+        <v>0.857</v>
       </c>
     </row>
     <row r="79" spans="1:8">
       <c r="A79" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B79" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C79">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D79">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E79">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F79">
-        <v>0.25</v>
+        <v>1.5</v>
       </c>
       <c r="G79">
-        <v>0.3</v>
+        <v>0.667</v>
       </c>
       <c r="H79">
-        <v>0.273</v>
+        <v>0.923</v>
       </c>
     </row>
     <row r="80" spans="1:8">
       <c r="A80" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B80" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C80">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="D80">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E80">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F80">
-        <v>0.25</v>
+        <v>0.727</v>
       </c>
       <c r="G80">
-        <v>1</v>
+        <v>0.889</v>
       </c>
       <c r="H80">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="81" spans="1:8">
       <c r="A81" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B81" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C81">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D81">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E81">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F81">
-        <v>0.462</v>
+        <v>0.7</v>
       </c>
       <c r="G81">
-        <v>0.6</v>
+        <v>0.778</v>
       </c>
       <c r="H81">
-        <v>0.522</v>
+        <v>0.737</v>
       </c>
     </row>
     <row r="82" spans="1:8">
       <c r="A82" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B82" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C82">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="D82">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E82">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F82">
-        <v>0.241</v>
+        <v>0.2</v>
       </c>
       <c r="G82">
-        <v>0.7</v>
+        <v>0.222</v>
       </c>
       <c r="H82">
-        <v>0.359</v>
+        <v>0.21</v>
       </c>
     </row>
     <row r="83" spans="1:8">
@@ -3416,25 +3422,25 @@
         <v>26</v>
       </c>
       <c r="B83" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C83">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="D83">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E83">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F83">
-        <v>0.412</v>
+        <v>1</v>
       </c>
       <c r="G83">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="H83">
-        <v>0.519</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84" spans="1:8">
@@ -3442,25 +3448,25 @@
         <v>26</v>
       </c>
       <c r="B84" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C84">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="D84">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E84">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F84">
-        <v>0</v>
+        <v>0.727</v>
       </c>
       <c r="G84">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H84">
-        <v>0</v>
+        <v>0.842</v>
       </c>
     </row>
     <row r="85" spans="1:8">
@@ -3468,181 +3474,181 @@
         <v>26</v>
       </c>
       <c r="B85" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C85">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D85">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E85">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F85">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G85">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H85">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:8">
       <c r="A86" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B86" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C86">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D86">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E86">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F86">
-        <v>0.2</v>
+        <v>0.667</v>
       </c>
       <c r="G86">
-        <v>0.286</v>
+        <v>0.5</v>
       </c>
       <c r="H86">
-        <v>0.235</v>
+        <v>0.572</v>
       </c>
     </row>
     <row r="87" spans="1:8">
       <c r="A87" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B87" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C87">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="D87">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E87">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F87">
-        <v>0.098</v>
+        <v>1.143</v>
       </c>
       <c r="G87">
-        <v>0.571</v>
+        <v>1</v>
       </c>
       <c r="H87">
-        <v>0.167</v>
+        <v>1.067</v>
       </c>
     </row>
     <row r="88" spans="1:8">
       <c r="A88" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B88" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C88">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D88">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E88">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F88">
-        <v>0.2</v>
+        <v>1.25</v>
       </c>
       <c r="G88">
-        <v>0.286</v>
+        <v>0.625</v>
       </c>
       <c r="H88">
-        <v>0.235</v>
+        <v>0.833</v>
       </c>
     </row>
     <row r="89" spans="1:8">
       <c r="A89" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B89" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C89">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D89">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E89">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F89">
-        <v>0.4</v>
+        <v>1.25</v>
       </c>
       <c r="G89">
-        <v>0.571</v>
+        <v>0.625</v>
       </c>
       <c r="H89">
-        <v>0.47</v>
+        <v>0.833</v>
       </c>
     </row>
     <row r="90" spans="1:8">
       <c r="A90" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B90" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C90">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="D90">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E90">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F90">
-        <v>0.3</v>
+        <v>1.25</v>
       </c>
       <c r="G90">
-        <v>0.429</v>
+        <v>0.625</v>
       </c>
       <c r="H90">
-        <v>0.353</v>
+        <v>0.833</v>
       </c>
     </row>
     <row r="91" spans="1:8">
       <c r="A91" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B91" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C91">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D91">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E91">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F91">
-        <v>0.143</v>
+        <v>1.333</v>
       </c>
       <c r="G91">
-        <v>0.143</v>
+        <v>0.5</v>
       </c>
       <c r="H91">
-        <v>0.143</v>
+        <v>0.727</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -3650,206 +3656,934 @@
         <v>27</v>
       </c>
       <c r="B92" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C92">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="D92">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E92">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F92">
-        <v>0.079</v>
+        <v>0.357</v>
       </c>
       <c r="G92">
-        <v>0.429</v>
+        <v>0.5</v>
       </c>
       <c r="H92">
-        <v>0.133</v>
+        <v>0.417</v>
       </c>
     </row>
     <row r="93" spans="1:8">
       <c r="A93" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B93" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C93">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="D93">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E93">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F93">
-        <v>0.909</v>
+        <v>0.146</v>
       </c>
       <c r="G93">
-        <v>0.909</v>
+        <v>0.6</v>
       </c>
       <c r="H93">
-        <v>0.909</v>
+        <v>0.235</v>
       </c>
     </row>
     <row r="94" spans="1:8">
       <c r="A94" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B94" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C94">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D94">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E94">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F94">
-        <v>0.909</v>
+        <v>0.143</v>
       </c>
       <c r="G94">
-        <v>0.909</v>
+        <v>0.2</v>
       </c>
       <c r="H94">
-        <v>0.909</v>
+        <v>0.167</v>
       </c>
     </row>
     <row r="95" spans="1:8">
       <c r="A95" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B95" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C95">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D95">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E95">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F95">
-        <v>0.909</v>
+        <v>0.4</v>
       </c>
       <c r="G95">
-        <v>0.909</v>
+        <v>0.6</v>
       </c>
       <c r="H95">
-        <v>0.909</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="96" spans="1:8">
       <c r="A96" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B96" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C96">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="D96">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E96">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F96">
-        <v>0.818</v>
+        <v>0.348</v>
       </c>
       <c r="G96">
-        <v>0.818</v>
+        <v>0.8</v>
       </c>
       <c r="H96">
-        <v>0.818</v>
+        <v>0.485</v>
       </c>
     </row>
     <row r="97" spans="1:8">
       <c r="A97" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B97" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C97">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D97">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E97">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F97">
-        <v>0.909</v>
+        <v>0.833</v>
       </c>
       <c r="G97">
-        <v>0.909</v>
+        <v>0.5</v>
       </c>
       <c r="H97">
-        <v>0.909</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="98" spans="1:8">
       <c r="A98" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B98" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C98">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D98">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E98">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="F98">
-        <v>1</v>
+        <v>0.182</v>
       </c>
       <c r="G98">
-        <v>0.818</v>
+        <v>0.2</v>
       </c>
       <c r="H98">
-        <v>0.9</v>
+        <v>0.191</v>
       </c>
     </row>
     <row r="99" spans="1:8">
       <c r="A99" t="s">
+        <v>27</v>
+      </c>
+      <c r="B99" t="s">
+        <v>16</v>
+      </c>
+      <c r="C99">
+        <v>15</v>
+      </c>
+      <c r="D99">
+        <v>10</v>
+      </c>
+      <c r="E99">
+        <v>5</v>
+      </c>
+      <c r="F99">
+        <v>0.333</v>
+      </c>
+      <c r="G99">
+        <v>0.5</v>
+      </c>
+      <c r="H99">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8">
+      <c r="A100" t="s">
+        <v>27</v>
+      </c>
+      <c r="B100" t="s">
+        <v>17</v>
+      </c>
+      <c r="C100">
+        <v>20</v>
+      </c>
+      <c r="D100">
+        <v>10</v>
+      </c>
+      <c r="E100">
+        <v>4</v>
+      </c>
+      <c r="F100">
+        <v>0.2</v>
+      </c>
+      <c r="G100">
+        <v>0.4</v>
+      </c>
+      <c r="H100">
+        <v>0.267</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8">
+      <c r="A101" t="s">
         <v>28</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B101" t="s">
+        <v>9</v>
+      </c>
+      <c r="C101">
+        <v>12</v>
+      </c>
+      <c r="D101">
+        <v>10</v>
+      </c>
+      <c r="E101">
+        <v>3</v>
+      </c>
+      <c r="F101">
+        <v>0.25</v>
+      </c>
+      <c r="G101">
+        <v>0.3</v>
+      </c>
+      <c r="H101">
+        <v>0.273</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8">
+      <c r="A102" t="s">
+        <v>28</v>
+      </c>
+      <c r="B102" t="s">
+        <v>10</v>
+      </c>
+      <c r="C102">
+        <v>40</v>
+      </c>
+      <c r="D102">
+        <v>10</v>
+      </c>
+      <c r="E102">
+        <v>10</v>
+      </c>
+      <c r="F102">
+        <v>0.25</v>
+      </c>
+      <c r="G102">
+        <v>1</v>
+      </c>
+      <c r="H102">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8">
+      <c r="A103" t="s">
+        <v>28</v>
+      </c>
+      <c r="B103" t="s">
+        <v>11</v>
+      </c>
+      <c r="C103">
+        <v>13</v>
+      </c>
+      <c r="D103">
+        <v>10</v>
+      </c>
+      <c r="E103">
+        <v>6</v>
+      </c>
+      <c r="F103">
+        <v>0.462</v>
+      </c>
+      <c r="G103">
+        <v>0.6</v>
+      </c>
+      <c r="H103">
+        <v>0.522</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8">
+      <c r="A104" t="s">
+        <v>28</v>
+      </c>
+      <c r="B104" t="s">
+        <v>12</v>
+      </c>
+      <c r="C104">
+        <v>29</v>
+      </c>
+      <c r="D104">
+        <v>10</v>
+      </c>
+      <c r="E104">
+        <v>7</v>
+      </c>
+      <c r="F104">
+        <v>0.241</v>
+      </c>
+      <c r="G104">
+        <v>0.7</v>
+      </c>
+      <c r="H104">
+        <v>0.359</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8">
+      <c r="A105" t="s">
+        <v>28</v>
+      </c>
+      <c r="B105" t="s">
+        <v>13</v>
+      </c>
+      <c r="C105">
+        <v>17</v>
+      </c>
+      <c r="D105">
+        <v>10</v>
+      </c>
+      <c r="E105">
+        <v>7</v>
+      </c>
+      <c r="F105">
+        <v>0.412</v>
+      </c>
+      <c r="G105">
+        <v>0.7</v>
+      </c>
+      <c r="H105">
+        <v>0.519</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8">
+      <c r="A106" t="s">
+        <v>28</v>
+      </c>
+      <c r="B106" t="s">
+        <v>14</v>
+      </c>
+      <c r="C106">
+        <v>3</v>
+      </c>
+      <c r="D106">
+        <v>10</v>
+      </c>
+      <c r="E106">
+        <v>0</v>
+      </c>
+      <c r="F106">
+        <v>0</v>
+      </c>
+      <c r="G106">
+        <v>0</v>
+      </c>
+      <c r="H106">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8">
+      <c r="A107" t="s">
+        <v>28</v>
+      </c>
+      <c r="B107" t="s">
         <v>15</v>
       </c>
-      <c r="C99">
+      <c r="C107">
+        <v>4</v>
+      </c>
+      <c r="D107">
+        <v>10</v>
+      </c>
+      <c r="E107">
+        <v>0</v>
+      </c>
+      <c r="F107">
+        <v>0</v>
+      </c>
+      <c r="G107">
+        <v>0</v>
+      </c>
+      <c r="H107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8">
+      <c r="A108" t="s">
+        <v>28</v>
+      </c>
+      <c r="B108" t="s">
+        <v>16</v>
+      </c>
+      <c r="C108">
+        <v>9</v>
+      </c>
+      <c r="D108">
+        <v>10</v>
+      </c>
+      <c r="E108">
+        <v>3</v>
+      </c>
+      <c r="F108">
+        <v>0.333</v>
+      </c>
+      <c r="G108">
+        <v>0.3</v>
+      </c>
+      <c r="H108">
+        <v>0.316</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8">
+      <c r="A109" t="s">
+        <v>28</v>
+      </c>
+      <c r="B109" t="s">
+        <v>17</v>
+      </c>
+      <c r="C109">
+        <v>3</v>
+      </c>
+      <c r="D109">
+        <v>10</v>
+      </c>
+      <c r="E109">
+        <v>0</v>
+      </c>
+      <c r="F109">
+        <v>0</v>
+      </c>
+      <c r="G109">
+        <v>0</v>
+      </c>
+      <c r="H109">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8">
+      <c r="A110" t="s">
+        <v>29</v>
+      </c>
+      <c r="B110" t="s">
+        <v>9</v>
+      </c>
+      <c r="C110">
+        <v>10</v>
+      </c>
+      <c r="D110">
+        <v>7</v>
+      </c>
+      <c r="E110">
+        <v>2</v>
+      </c>
+      <c r="F110">
+        <v>0.2</v>
+      </c>
+      <c r="G110">
+        <v>0.286</v>
+      </c>
+      <c r="H110">
+        <v>0.235</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8">
+      <c r="A111" t="s">
+        <v>29</v>
+      </c>
+      <c r="B111" t="s">
+        <v>10</v>
+      </c>
+      <c r="C111">
+        <v>41</v>
+      </c>
+      <c r="D111">
+        <v>7</v>
+      </c>
+      <c r="E111">
+        <v>4</v>
+      </c>
+      <c r="F111">
+        <v>0.098</v>
+      </c>
+      <c r="G111">
+        <v>0.571</v>
+      </c>
+      <c r="H111">
+        <v>0.167</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8">
+      <c r="A112" t="s">
+        <v>29</v>
+      </c>
+      <c r="B112" t="s">
         <v>11</v>
       </c>
-      <c r="D99">
+      <c r="C112">
+        <v>10</v>
+      </c>
+      <c r="D112">
+        <v>7</v>
+      </c>
+      <c r="E112">
+        <v>2</v>
+      </c>
+      <c r="F112">
+        <v>0.2</v>
+      </c>
+      <c r="G112">
+        <v>0.286</v>
+      </c>
+      <c r="H112">
+        <v>0.235</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8">
+      <c r="A113" t="s">
+        <v>29</v>
+      </c>
+      <c r="B113" t="s">
+        <v>12</v>
+      </c>
+      <c r="C113">
+        <v>10</v>
+      </c>
+      <c r="D113">
+        <v>7</v>
+      </c>
+      <c r="E113">
+        <v>4</v>
+      </c>
+      <c r="F113">
+        <v>0.4</v>
+      </c>
+      <c r="G113">
+        <v>0.571</v>
+      </c>
+      <c r="H113">
+        <v>0.47</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8">
+      <c r="A114" t="s">
+        <v>29</v>
+      </c>
+      <c r="B114" t="s">
+        <v>13</v>
+      </c>
+      <c r="C114">
+        <v>10</v>
+      </c>
+      <c r="D114">
+        <v>7</v>
+      </c>
+      <c r="E114">
+        <v>3</v>
+      </c>
+      <c r="F114">
+        <v>0.3</v>
+      </c>
+      <c r="G114">
+        <v>0.429</v>
+      </c>
+      <c r="H114">
+        <v>0.353</v>
+      </c>
+    </row>
+    <row r="115" spans="1:8">
+      <c r="A115" t="s">
+        <v>29</v>
+      </c>
+      <c r="B115" t="s">
+        <v>14</v>
+      </c>
+      <c r="C115">
+        <v>7</v>
+      </c>
+      <c r="D115">
+        <v>7</v>
+      </c>
+      <c r="E115">
+        <v>1</v>
+      </c>
+      <c r="F115">
+        <v>0.143</v>
+      </c>
+      <c r="G115">
+        <v>0.143</v>
+      </c>
+      <c r="H115">
+        <v>0.143</v>
+      </c>
+    </row>
+    <row r="116" spans="1:8">
+      <c r="A116" t="s">
+        <v>29</v>
+      </c>
+      <c r="B116" t="s">
+        <v>15</v>
+      </c>
+      <c r="C116">
+        <v>8</v>
+      </c>
+      <c r="D116">
+        <v>7</v>
+      </c>
+      <c r="E116">
+        <v>2</v>
+      </c>
+      <c r="F116">
+        <v>0.25</v>
+      </c>
+      <c r="G116">
+        <v>0.286</v>
+      </c>
+      <c r="H116">
+        <v>0.267</v>
+      </c>
+    </row>
+    <row r="117" spans="1:8">
+      <c r="A117" t="s">
+        <v>29</v>
+      </c>
+      <c r="B117" t="s">
+        <v>16</v>
+      </c>
+      <c r="C117">
+        <v>7</v>
+      </c>
+      <c r="D117">
+        <v>7</v>
+      </c>
+      <c r="E117">
+        <v>0</v>
+      </c>
+      <c r="F117">
+        <v>0</v>
+      </c>
+      <c r="G117">
+        <v>0</v>
+      </c>
+      <c r="H117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:8">
+      <c r="A118" t="s">
+        <v>29</v>
+      </c>
+      <c r="B118" t="s">
+        <v>17</v>
+      </c>
+      <c r="C118">
+        <v>38</v>
+      </c>
+      <c r="D118">
+        <v>7</v>
+      </c>
+      <c r="E118">
+        <v>3</v>
+      </c>
+      <c r="F118">
+        <v>0.079</v>
+      </c>
+      <c r="G118">
+        <v>0.429</v>
+      </c>
+      <c r="H118">
+        <v>0.133</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8">
+      <c r="A119" t="s">
+        <v>30</v>
+      </c>
+      <c r="B119" t="s">
+        <v>9</v>
+      </c>
+      <c r="C119">
         <v>11</v>
       </c>
-      <c r="E99">
-        <v>9</v>
-      </c>
-      <c r="F99">
+      <c r="D119">
+        <v>11</v>
+      </c>
+      <c r="E119">
+        <v>10</v>
+      </c>
+      <c r="F119">
+        <v>0.909</v>
+      </c>
+      <c r="G119">
+        <v>0.909</v>
+      </c>
+      <c r="H119">
+        <v>0.909</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8">
+      <c r="A120" t="s">
+        <v>30</v>
+      </c>
+      <c r="B120" t="s">
+        <v>10</v>
+      </c>
+      <c r="C120">
+        <v>11</v>
+      </c>
+      <c r="D120">
+        <v>11</v>
+      </c>
+      <c r="E120">
+        <v>10</v>
+      </c>
+      <c r="F120">
+        <v>0.909</v>
+      </c>
+      <c r="G120">
+        <v>0.909</v>
+      </c>
+      <c r="H120">
+        <v>0.909</v>
+      </c>
+    </row>
+    <row r="121" spans="1:8">
+      <c r="A121" t="s">
+        <v>30</v>
+      </c>
+      <c r="B121" t="s">
+        <v>11</v>
+      </c>
+      <c r="C121">
+        <v>11</v>
+      </c>
+      <c r="D121">
+        <v>11</v>
+      </c>
+      <c r="E121">
+        <v>10</v>
+      </c>
+      <c r="F121">
+        <v>0.909</v>
+      </c>
+      <c r="G121">
+        <v>0.909</v>
+      </c>
+      <c r="H121">
+        <v>0.909</v>
+      </c>
+    </row>
+    <row r="122" spans="1:8">
+      <c r="A122" t="s">
+        <v>30</v>
+      </c>
+      <c r="B122" t="s">
+        <v>12</v>
+      </c>
+      <c r="C122">
+        <v>11</v>
+      </c>
+      <c r="D122">
+        <v>11</v>
+      </c>
+      <c r="E122">
+        <v>9</v>
+      </c>
+      <c r="F122">
         <v>0.818</v>
       </c>
-      <c r="G99">
+      <c r="G122">
         <v>0.818</v>
       </c>
-      <c r="H99">
+      <c r="H122">
+        <v>0.818</v>
+      </c>
+    </row>
+    <row r="123" spans="1:8">
+      <c r="A123" t="s">
+        <v>30</v>
+      </c>
+      <c r="B123" t="s">
+        <v>13</v>
+      </c>
+      <c r="C123">
+        <v>11</v>
+      </c>
+      <c r="D123">
+        <v>11</v>
+      </c>
+      <c r="E123">
+        <v>10</v>
+      </c>
+      <c r="F123">
+        <v>0.909</v>
+      </c>
+      <c r="G123">
+        <v>0.909</v>
+      </c>
+      <c r="H123">
+        <v>0.909</v>
+      </c>
+    </row>
+    <row r="124" spans="1:8">
+      <c r="A124" t="s">
+        <v>30</v>
+      </c>
+      <c r="B124" t="s">
+        <v>14</v>
+      </c>
+      <c r="C124">
+        <v>9</v>
+      </c>
+      <c r="D124">
+        <v>11</v>
+      </c>
+      <c r="E124">
+        <v>9</v>
+      </c>
+      <c r="F124">
+        <v>1</v>
+      </c>
+      <c r="G124">
+        <v>0.818</v>
+      </c>
+      <c r="H124">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="125" spans="1:8">
+      <c r="A125" t="s">
+        <v>30</v>
+      </c>
+      <c r="B125" t="s">
+        <v>15</v>
+      </c>
+      <c r="C125">
+        <v>9</v>
+      </c>
+      <c r="D125">
+        <v>11</v>
+      </c>
+      <c r="E125">
+        <v>9</v>
+      </c>
+      <c r="F125">
+        <v>1</v>
+      </c>
+      <c r="G125">
+        <v>0.818</v>
+      </c>
+      <c r="H125">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="126" spans="1:8">
+      <c r="A126" t="s">
+        <v>30</v>
+      </c>
+      <c r="B126" t="s">
+        <v>16</v>
+      </c>
+      <c r="C126">
+        <v>9</v>
+      </c>
+      <c r="D126">
+        <v>11</v>
+      </c>
+      <c r="E126">
+        <v>6</v>
+      </c>
+      <c r="F126">
+        <v>0.667</v>
+      </c>
+      <c r="G126">
+        <v>0.545</v>
+      </c>
+      <c r="H126">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="127" spans="1:8">
+      <c r="A127" t="s">
+        <v>30</v>
+      </c>
+      <c r="B127" t="s">
+        <v>17</v>
+      </c>
+      <c r="C127">
+        <v>11</v>
+      </c>
+      <c r="D127">
+        <v>11</v>
+      </c>
+      <c r="E127">
+        <v>9</v>
+      </c>
+      <c r="F127">
+        <v>0.818</v>
+      </c>
+      <c r="G127">
+        <v>0.818</v>
+      </c>
+      <c r="H127">
         <v>0.818</v>
       </c>
     </row>

</xml_diff>